<commit_message>
docs: record final NutFT validation
</commit_message>
<xml_diff>
--- a/outputs/01a015ae-ab4f-7202-8d77-0679917a61c4/nutft-platform-validation.xlsx
+++ b/outputs/01a015ae-ab4f-7202-8d77-0679917a61c4/nutft-platform-validation.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf945b1e55c2c4fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R4a85013653944c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="3" r:id="R39d94d84154c4d93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="Rf28fb64289b94ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="5" r:id="R9d6c6df449654029"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4431733f049847bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="Raafce013bfeb41d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="3" r:id="R07e7b89b191643fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R8f235cbca54147e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="5" r:id="R1c78e9095a7a4ab8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -594,7 +594,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Breno" id="{3C0E0E67-8D8E-47AB-895E-5A1473C627F6}"/>
+  <xltc:person displayName="Breno" id="{48E8FDB5-6176-4F8F-97C1-784795BAF667}"/>
 </xltc:personList>
 </file>
 
@@ -637,7 +637,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DefectsTable" displayName="DefectsTable" ref="A5:K44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DefectsTable" displayName="DefectsTable" ref="A5:K45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Severity"/>
@@ -1066,7 +1066,7 @@
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="47" t="str">
-        <x:v>Current gate: COMPLETE. All 78 cataloged user stories and 26 protocol requirements pass final automated/browser evidence. All in-scope defects are verified; D-018 tracks six pre-existing optional art/font checks.</x:v>
+        <x:v>Current gate: COMPLETE. All 78 cataloged user stories and 26 protocol requirements pass final automated/browser evidence. All 39 in-scope defects are verified; D-018 tracks six pre-existing optional art/font checks.</x:v>
       </x:c>
       <x:c r="B11" s="45"/>
       <x:c r="C11" s="45"/>
@@ -1120,7 +1120,7 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="C14" s="45" t="str">
-        <x:v>78 stories · 26 protocol rows · 39 defects</x:v>
+        <x:v>78 stories · 26 protocol rows · 40 defects</x:v>
       </x:c>
       <x:c r="D14" s="45" t="str">
         <x:v>None</x:v>
@@ -1172,7 +1172,7 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="C16" s="45" t="str">
-        <x:v>13 atomic commits with regressions</x:v>
+        <x:v>14 atomic commits with regressions</x:v>
       </x:c>
       <x:c r="D16" s="45" t="str">
         <x:v>None</x:v>
@@ -1213,7 +1213,7 @@
         <x:v>#4</x:v>
       </x:c>
       <x:c r="H17" s="45" t="str">
-        <x:v>315 JS + two browser matrices</x:v>
+        <x:v>316 JS + two browser matrices</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4970,7 +4970,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a964a8b4a4a4c39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ccb882d1a184b20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5653,7 +5653,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b02796a8a684760"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25ed1954041041d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7159,32 +7159,67 @@
         <x:v>Verified</x:v>
       </x:c>
     </x:row>
+    <x:row r="45" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A45" s="69" t="str">
+        <x:v>D-040</x:v>
+      </x:c>
+      <x:c r="B45" s="69" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="C45" s="69" t="str">
+        <x:v>Mint configuration</x:v>
+      </x:c>
+      <x:c r="D45" s="69" t="str">
+        <x:v>A persisted mint could restart under a different census, collection, or catalog URI and split CardBinding compatibility.</x:v>
+      </x:c>
+      <x:c r="E45" s="69" t="str">
+        <x:v>Create database, restart with changed catalog URI.</x:v>
+      </x:c>
+      <x:c r="F45" s="69" t="str">
+        <x:v>Refuse boot and close the database handle.</x:v>
+      </x:c>
+      <x:c r="G45" s="69" t="str">
+        <x:v>Persisted keys/state were reused with a new binding namespace.</x:v>
+      </x:c>
+      <x:c r="H45" s="69" t="str">
+        <x:v>Remote branch regression review</x:v>
+      </x:c>
+      <x:c r="I45" s="69" t="str">
+        <x:v>Focused restart/config test</x:v>
+      </x:c>
+      <x:c r="J45" s="69" t="str">
+        <x:v>bb1731c</x:v>
+      </x:c>
+      <x:c r="K45" s="69" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K44">
+  <x:conditionalFormatting sqref="K6:K45">
     <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Pass"/>
     <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="Fail"/>
     <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="Blocked"/>
     <x:cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="Not Run"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B6:B44">
+  <x:conditionalFormatting sqref="B6:B45">
     <x:cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Critical"/>
     <x:cfRule type="containsText" dxfId="13" priority="6" operator="containsText" text="High"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B6:B44">
+    <x:dataValidation type="list" sqref="B6:B45">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K6:K44">
+    <x:dataValidation type="list" sqref="K6:K45">
       <x:formula1>"Open,In Progress,Fixed,Verified,Triaged,Won't Fix"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R870630f5b7164a8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R511f5f9f293348c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7449,7 +7484,7 @@
         <x:v>D-001</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
+    <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A10" s="69" t="str">
         <x:v>RUN-005</x:v>
       </x:c>
@@ -7466,7 +7501,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="F10" s="71" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="71" t="n">
         <x:v>0</x:v>
@@ -7475,10 +7510,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="69" t="str">
-        <x:v>Output openings, URI validation, two-wallet transfer/import, backup/restore, lost-response recovery, restart persistence, DLEQ, P2BK, binding, checkstate, swap/melt rejection</x:v>
+        <x:v>Output openings, URI/config validation, two-wallet transfer/import, backup/restore, lost-response recovery, restart persistence, DLEQ, P2BK, binding, checkstate, swap/melt rejection</x:v>
       </x:c>
       <x:c r="J10" s="69" t="str">
-        <x:v>Final branch b1fd2bf</x:v>
+        <x:v>Final branch</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -7498,7 +7533,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="F11" s="71" t="n">
-        <x:v>315</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="G11" s="71" t="n">
         <x:v>0</x:v>
@@ -7507,7 +7542,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="69" t="str">
-        <x:v>315 tests passed in 12.1s</x:v>
+        <x:v>316 tests passed</x:v>
       </x:c>
       <x:c r="J11" s="69" t="str">
         <x:v>Engine, client, transport, online play, ladder, Cashu/NutFT, card waves, QR, and crypto</x:v>
@@ -7654,7 +7689,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05016cc48cb84128"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71b8d5d96c1e4df4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>